<commit_message>
feat: Elder Dashboard rebuild matching 5 reference images — Governance, Monthly Submission, Priest Review, Risk & Audit tabs
</commit_message>
<xml_diff>
--- a/docs/design/Elder_dashboard_ideas.xlsx
+++ b/docs/design/Elder_dashboard_ideas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goscorpty-my.sharepoint.com/personal/jermainem_goscor_co_za/Documents/Documents/OAC/KasBoek/jw-cashbook-v4/docs/design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{B92DEF30-A178-4046-A2CE-B6824D1042C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6374C77E-1FEB-445A-82AE-4E2C1C4B1DF7}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{B92DEF30-A178-4046-A2CE-B6824D1042C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{259F08CE-FDBD-482B-BF8A-02B144E46276}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{96E2BB65-FE70-4926-ACE7-07AFBD5AA238}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
   <si>
     <t>Elder Dashboard ideas</t>
   </si>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t>Eldership Total</t>
+  </si>
+  <si>
+    <t>+          Bomont</t>
+  </si>
+  <si>
+    <t>+        Newclare</t>
   </si>
 </sst>
 </file>
@@ -1947,16 +1953,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>542924</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>438149</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>314324</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>295274</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1971,7 +1977,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="542924" y="6848475"/>
+          <a:off x="11163299" y="6886575"/>
           <a:ext cx="1685925" cy="1000125"/>
         </a:xfrm>
         <a:prstGeom prst="teardrop">
@@ -2849,7 +2855,7 @@
         <v>3</v>
       </c>
       <c r="E35" s="36" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="F35" s="63">
         <f>SUM(F36:F40)</f>
@@ -2876,7 +2882,7 @@
         <v>11902</v>
       </c>
     </row>
-    <row r="36" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E36" s="41" t="s">
         <v>37</v>
       </c>
@@ -2900,7 +2906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E37" s="41" t="s">
         <v>38</v>
       </c>
@@ -2924,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E38" s="41" t="s">
         <v>39</v>
       </c>
@@ -2949,7 +2955,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="39" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E39" s="41" t="s">
         <v>40</v>
       </c>
@@ -2974,7 +2980,7 @@
         <v>11452</v>
       </c>
     </row>
-    <row r="40" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E40" s="41" t="s">
         <v>41</v>
       </c>
@@ -2998,7 +3004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="4:11" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E41" s="41" t="s">
         <v>52</v>
       </c>
@@ -3029,7 +3035,7 @@
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.25">
       <c r="E42" s="36" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="F42" s="53">
         <f>SUM(F43:F47)</f>
@@ -3056,7 +3062,7 @@
         <v>8944</v>
       </c>
     </row>
-    <row r="43" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E43" s="41" t="s">
         <v>42</v>
       </c>
@@ -3081,7 +3087,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E44" s="41" t="s">
         <v>43</v>
       </c>
@@ -3106,7 +3112,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="45" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E45" s="41" t="s">
         <v>44</v>
       </c>
@@ -3131,7 +3137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E46" s="41" t="s">
         <v>45</v>
       </c>
@@ -3156,7 +3162,7 @@
         <v>8009</v>
       </c>
     </row>
-    <row r="47" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:11" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="E47" s="41" t="s">
         <v>46</v>
       </c>
@@ -3181,7 +3187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="4:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:11" collapsed="1" x14ac:dyDescent="0.25">
       <c r="E48" s="41" t="s">
         <v>52</v>
       </c>

</xml_diff>